<commit_message>
Demuestra en los ejemplos la unicidad contra el catálogo
Las incidencias VAL-UNI-003 y VAL-UNI-004 del archivo de ejemplo solo
mostraban filas chocando entre sí dentro del archivo. El caso que agregó
revisarUnicidadContraCatalogo —una sola fila que choca contra algo que ya
está cargado— no se podía armar a mano, porque el catálogo se genera al
azar en cada sesión y un código fijo en el .xlsx no tenía con qué chocar.

El catálogo arranca ahora con una fila ancla fija —código 1001293, Robert
Bosch México, GTIN 07500001234563 en Presentación · Caja máster · 24—
además de las 182 aleatorias. La fila 19 de Importar-incompletos.xlsx
trae ese mismo GTIN con alcance Producto y otro proveedor, de modo que la
incidencia se levanta contra el catálogo, no contra otra fila del
archivo, y el resultado es idéntico en cualquier sesión.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JJrqS6Z27X2jyr3npi3vA3
</commit_message>
<xml_diff>
--- a/ejemplos/Importar-incompletos.xlsx
+++ b/ejemplos/Importar-incompletos.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1124,22 +1124,24 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="n">
-        <v>1001000</v>
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>1001293</t>
+        </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Dana Transmisiones</t>
+          <t>Hella Iluminación</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>No GS1</t>
+          <t>GS1</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>PROP-C-200</t>
+          <t>07500001234563</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1163,37 +1165,75 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
+        <v>1001000</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Dana Transmisiones</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>No GS1</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>PROP-C-200</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Producto</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
         <v>1023711</v>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>Delphi Technologies</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>No GS1</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>PROP-C-200</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>Presentación</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>Pallet</t>
         </is>
       </c>
-      <c r="G20" t="n">
+      <c r="G21" t="n">
         <v>96</v>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="H21" t="inlineStr">
         <is>
           <t>Activo</t>
         </is>

</xml_diff>